<commit_message>
docs(task_submission): 同步自验证报告中的 commit 基线
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/task_submission/2.1_精度自验证报告.xlsx
+++ b/task_submission/2.1_精度自验证报告.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -561,7 +561,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>96818d4f</t>
+          <t>72bb444f</t>
         </is>
       </c>
       <c r="F3" s="5" t="n"/>
@@ -1102,7 +1102,7 @@
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>环境与复现：source /usr/local/Ascend/cann/set_env.sh；export LD_LIBRARY_PATH=${ASCEND_HOME_PATH}/opp/vendors/custom_transformer/op_api/lib:${LD_LIBRARY_PATH}；全量精度 /root/backup/full_prec_runner；example：bash build.sh --run_example turbo_quant_attention_score eager cust --vendor_name=custom --soc=ascend910b --experimental。仓 https://gitcode.com/sun_king_poem/ops-transformer 分支 feat/turbo_quant_attention_score commit 96818d4f。截图粘贴到「Ascend截图」列对应单元格；本算子无 TBE，「TBE截图」填无 TBE。</t>
+          <t>环境与复现：source /usr/local/Ascend/cann/set_env.sh；export LD_LIBRARY_PATH=${ASCEND_HOME_PATH}/opp/vendors/custom_transformer/op_api/lib:${LD_LIBRARY_PATH}；全量精度 /root/backup/full_prec_runner；example：bash build.sh --run_example turbo_quant_attention_score eager cust --vendor_name=custom --soc=ascend910b --experimental。仓 https://gitcode.com/sun_king_poem/ops-transformer 分支 feat/turbo_quant_attention_score commit 72bb444f。截图粘贴到「Ascend截图」列对应单元格；本算子无 TBE，「TBE截图」填无 TBE。</t>
         </is>
       </c>
       <c r="B15" s="6" t="n"/>
@@ -1115,11 +1115,6 @@
       <c r="I15" s="6" t="n"/>
       <c r="J15" s="5" t="n"/>
     </row>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:J1"/>

</xml_diff>